<commit_message>
Update course list and remove reference files
</commit_message>
<xml_diff>
--- a/Course List/Course list.xlsx
+++ b/Course List/Course list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\Stats\code\Bot\Course List\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7FD6BE-A8AE-458C-8ECD-E8E8BFBCF231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFAB2FC-2B02-46C5-8551-49C5817CF8CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NCUFN" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="239">
   <si>
     <t>StudentID</t>
   </si>
@@ -34,10 +34,184 @@
     <t>Password</t>
   </si>
   <si>
-    <t>符傳忠</t>
-  </si>
-  <si>
-    <t>110408547statistic</t>
+    <t>11050197</t>
+  </si>
+  <si>
+    <t>吳太惠</t>
+  </si>
+  <si>
+    <t>11140289</t>
+  </si>
+  <si>
+    <t>翁廣勝</t>
+  </si>
+  <si>
+    <t>11340171</t>
+  </si>
+  <si>
+    <t>劉雯惠</t>
+  </si>
+  <si>
+    <t>11340172</t>
+  </si>
+  <si>
+    <t>吳榮臻</t>
+  </si>
+  <si>
+    <t>11340173</t>
+  </si>
+  <si>
+    <t>潘順財</t>
+  </si>
+  <si>
+    <t>11340174</t>
+  </si>
+  <si>
+    <t>譚浩賢</t>
+  </si>
+  <si>
+    <t>11340175</t>
+  </si>
+  <si>
+    <t>沈書宇</t>
+  </si>
+  <si>
+    <t>11340179</t>
+  </si>
+  <si>
+    <t>中舘季来</t>
+  </si>
+  <si>
+    <t>11340180</t>
+  </si>
+  <si>
+    <t>月鑽</t>
+  </si>
+  <si>
+    <t>11340184</t>
+  </si>
+  <si>
+    <t>陳慧芳</t>
+  </si>
+  <si>
+    <t>11340188</t>
+  </si>
+  <si>
+    <t>邱曉涵</t>
+  </si>
+  <si>
+    <t>11340192</t>
+  </si>
+  <si>
+    <t>陳慧晶</t>
+  </si>
+  <si>
+    <t>11340197</t>
+  </si>
+  <si>
+    <t>濱中芽依</t>
+  </si>
+  <si>
+    <t>11340198</t>
+  </si>
+  <si>
+    <t>關川愛真</t>
+  </si>
+  <si>
+    <t>11340199</t>
+  </si>
+  <si>
+    <t>黄恩斯</t>
+  </si>
+  <si>
+    <t>11340201</t>
+  </si>
+  <si>
+    <t>任紹軒</t>
+  </si>
+  <si>
+    <t>11340209</t>
+  </si>
+  <si>
+    <t>陳義範</t>
+  </si>
+  <si>
+    <t>11340210</t>
+  </si>
+  <si>
+    <t>陳漢亮</t>
+  </si>
+  <si>
+    <t>11340215</t>
+  </si>
+  <si>
+    <t>馮明凱</t>
+  </si>
+  <si>
+    <t>11340217</t>
+  </si>
+  <si>
+    <t>葉明煜</t>
+  </si>
+  <si>
+    <t>11340219</t>
+  </si>
+  <si>
+    <t>蘇春福</t>
+  </si>
+  <si>
+    <t>11340220</t>
+  </si>
+  <si>
+    <t>上里苺葉</t>
+  </si>
+  <si>
+    <t>11340222</t>
+  </si>
+  <si>
+    <t>周榮仙</t>
+  </si>
+  <si>
+    <t>11340230</t>
+  </si>
+  <si>
+    <t>鐘怡柔</t>
+  </si>
+  <si>
+    <t>11340231</t>
+  </si>
+  <si>
+    <t>王祿康</t>
+  </si>
+  <si>
+    <t>11340232</t>
+  </si>
+  <si>
+    <t>李健明</t>
+  </si>
+  <si>
+    <t>11340233</t>
+  </si>
+  <si>
+    <t>鄧美玲</t>
+  </si>
+  <si>
+    <t>11340234</t>
+  </si>
+  <si>
+    <t>林麗燕</t>
+  </si>
+  <si>
+    <t>丁聖曦</t>
+  </si>
+  <si>
+    <t>藍宇皓</t>
+  </si>
+  <si>
+    <t>魏士凱</t>
+  </si>
+  <si>
+    <t>91111408527</t>
   </si>
   <si>
     <t>黃沛鈞</t>
@@ -46,7 +220,10 @@
     <t>112103011</t>
   </si>
   <si>
-    <t>林子元</t>
+    <t>唐瑄妤</t>
+  </si>
+  <si>
+    <t>tgs650730ARMY</t>
   </si>
   <si>
     <t>鄭煒騰</t>
@@ -64,7 +241,7 @@
     <t>李　琦</t>
   </si>
   <si>
-    <t>1134O8oo2</t>
+    <t>lee0413</t>
   </si>
   <si>
     <t>吳旻瑄</t>
@@ -76,15 +253,12 @@
     <t>陳欣琦</t>
   </si>
   <si>
-    <t>1141statdis</t>
+    <t>1142statdis</t>
   </si>
   <si>
     <t>吳芊嬅</t>
   </si>
   <si>
-    <t>113408005</t>
-  </si>
-  <si>
     <t>陳禹蓁</t>
   </si>
   <si>
@@ -94,12 +268,15 @@
     <t>余湘珍</t>
   </si>
   <si>
-    <t>密碼：113408008ncufn</t>
+    <t>113408008ncufn</t>
   </si>
   <si>
     <t>施宇晏</t>
   </si>
   <si>
+    <t>20080064</t>
+  </si>
+  <si>
     <t>賴瀅婕</t>
   </si>
   <si>
@@ -109,20 +286,17 @@
     <t>陳品晴</t>
   </si>
   <si>
-    <t>abcd12345</t>
+    <t>121231234</t>
   </si>
   <si>
     <t>黃子紜</t>
   </si>
   <si>
-    <t>113408012</t>
-  </si>
-  <si>
     <t>黃鈺玲</t>
   </si>
   <si>
-    <t>student: 黃鈺玲 113408015
-password: DomLyn2005</t>
+    <t>113408015 黃鈺玲
+password : domlyn0520</t>
   </si>
   <si>
     <t>廖施萍</t>
@@ -131,12 +305,6 @@
     <t>0192837465</t>
   </si>
   <si>
-    <t>簡睿宇</t>
-  </si>
-  <si>
-    <t>fstaticu3118</t>
-  </si>
-  <si>
     <t>陳珺豪</t>
   </si>
   <si>
@@ -152,6 +320,9 @@
     <t>陳友倫</t>
   </si>
   <si>
+    <t>113408020</t>
+  </si>
+  <si>
     <t>范毓恩</t>
   </si>
   <si>
@@ -167,52 +338,52 @@
     <t>曾亦呈</t>
   </si>
   <si>
+    <t>12345678</t>
+  </si>
+  <si>
+    <t>吳則澔</t>
+  </si>
+  <si>
+    <t>hao950430</t>
+  </si>
+  <si>
+    <t>余家聰</t>
+  </si>
+  <si>
+    <t>Password:3121243</t>
+  </si>
+  <si>
+    <t>吳黃暐博</t>
+  </si>
+  <si>
+    <t>曾怡瑄</t>
+  </si>
+  <si>
+    <t>statistic1142</t>
+  </si>
+  <si>
+    <t>林昱欣</t>
+  </si>
+  <si>
+    <t>wodemingzishilinyuxin</t>
+  </si>
+  <si>
+    <t>謝昀妃</t>
+  </si>
+  <si>
+    <t>Rr0958826491@</t>
+  </si>
+  <si>
+    <t>李雨芮</t>
+  </si>
+  <si>
     <t>123456789</t>
   </si>
   <si>
-    <t>吳則澔</t>
-  </si>
-  <si>
-    <t>hao950430</t>
-  </si>
-  <si>
-    <t>余家聰</t>
-  </si>
-  <si>
-    <t>Kachung1324</t>
-  </si>
-  <si>
-    <t>吳黃暐博</t>
-  </si>
-  <si>
-    <t>曾怡瑄</t>
-  </si>
-  <si>
-    <t>#Oo54360921</t>
-  </si>
-  <si>
-    <t>林昱欣</t>
-  </si>
-  <si>
-    <t>wodemingzishilinyuxin</t>
-  </si>
-  <si>
-    <t>謝昀妃</t>
-  </si>
-  <si>
-    <t>Rr0958826491@</t>
-  </si>
-  <si>
-    <t>李雨芮</t>
-  </si>
-  <si>
-    <t>Aa123456789</t>
-  </si>
-  <si>
     <t>洪向秀</t>
   </si>
   <si>
-    <t>hung20051006</t>
+    <t>JlplhQHi*5Iy</t>
   </si>
   <si>
     <t>楊于嫻</t>
@@ -224,7 +395,7 @@
     <t>姚怡如</t>
   </si>
   <si>
-    <t>lulu123123</t>
+    <t>lulu123</t>
   </si>
   <si>
     <t>胡瑜涵</t>
@@ -242,7 +413,7 @@
     <t>郭喜沛</t>
   </si>
   <si>
-    <t>密碼:fatguOzz0</t>
+    <t>0380</t>
   </si>
   <si>
     <t>羅翊恩</t>
@@ -266,25 +437,25 @@
     <t>吳玟</t>
   </si>
   <si>
-    <t>1304222www</t>
+    <t>130</t>
   </si>
   <si>
     <t>陳苡瑄</t>
   </si>
   <si>
-    <t>113408515wlk</t>
+    <t>113408515lyn</t>
   </si>
   <si>
     <t>涂筱嫻</t>
   </si>
   <si>
-    <t>a113408516</t>
+    <t>113408516</t>
   </si>
   <si>
     <t>江巽與</t>
   </si>
   <si>
-    <t>dofine@nicole</t>
+    <t>06100715</t>
   </si>
   <si>
     <t>王盈婷</t>
@@ -308,13 +479,13 @@
     <t>林謙愛</t>
   </si>
   <si>
-    <t>IRENE2005</t>
+    <t>Strawberry123</t>
   </si>
   <si>
     <t>許彩瑩</t>
   </si>
   <si>
-    <t>12345qwert</t>
+    <t>20051005</t>
   </si>
   <si>
     <t>王振諺</t>
@@ -347,199 +518,100 @@
     <t>張峻瑋</t>
   </si>
   <si>
-    <t>stat010154</t>
+    <t>100353</t>
   </si>
   <si>
     <t>陳奕翔</t>
   </si>
   <si>
-    <t>113408530</t>
-  </si>
-  <si>
-    <t>梁鈞傑</t>
-  </si>
-  <si>
-    <t>031206</t>
-  </si>
-  <si>
-    <t>林玄燁</t>
-  </si>
-  <si>
     <t>陳星碩</t>
   </si>
   <si>
-    <t>hsing113408533star</t>
-  </si>
-  <si>
     <t>陳宥軍</t>
   </si>
   <si>
-    <t>doilooklikeawhitemouse?</t>
-  </si>
-  <si>
     <t>許崴竣</t>
   </si>
   <si>
-    <t>dongyu1226</t>
-  </si>
-  <si>
     <t>謝岱凌</t>
   </si>
   <si>
-    <t>tailing0000</t>
-  </si>
-  <si>
-    <t>顏千茹</t>
-  </si>
-  <si>
-    <t>范芩蜜</t>
-  </si>
-  <si>
-    <t>潘又銘</t>
-  </si>
-  <si>
-    <t>陳思昀</t>
-  </si>
-  <si>
-    <t>方子妍</t>
+    <t>夏資喻</t>
   </si>
   <si>
     <t>黃泓瑜</t>
   </si>
   <si>
-    <t>0423116978</t>
+    <t>柯閔棨</t>
+  </si>
+  <si>
+    <t>王柏涵</t>
+  </si>
+  <si>
+    <t>葉錦徽</t>
   </si>
   <si>
     <t>計道揆</t>
   </si>
   <si>
-    <t>林冠妤</t>
-  </si>
-  <si>
-    <t>931220</t>
-  </si>
-  <si>
-    <t>徐榮萱</t>
-  </si>
-  <si>
-    <t>Mouo0205</t>
-  </si>
-  <si>
     <t>謝恩妮</t>
   </si>
   <si>
     <t>amber941108</t>
   </si>
   <si>
-    <t>曾翎琍</t>
-  </si>
-  <si>
-    <t>heidi0000</t>
-  </si>
-  <si>
     <t>蘇于婷</t>
   </si>
   <si>
-    <t>113409004dc</t>
-  </si>
-  <si>
-    <t>楊婕寧</t>
-  </si>
-  <si>
     <t>江子欣</t>
   </si>
   <si>
     <t>hsin24762</t>
   </si>
   <si>
-    <t>陳潔瑩</t>
-  </si>
-  <si>
-    <t>18179jy</t>
-  </si>
-  <si>
     <t>張秀麗</t>
   </si>
   <si>
-    <t>密碼 ： truongtule1009</t>
+    <t>tule240901</t>
   </si>
   <si>
     <t>賴小雨</t>
   </si>
   <si>
-    <t>CindeaCantik265</t>
-  </si>
-  <si>
-    <t>曾韋文</t>
-  </si>
-  <si>
     <t>周訓霆</t>
   </si>
   <si>
-    <t>Alanmcr7</t>
-  </si>
-  <si>
-    <t>葉栩呈</t>
-  </si>
-  <si>
-    <t>s10330910</t>
-  </si>
-  <si>
     <t>胡宸瑋</t>
   </si>
   <si>
-    <t>OAoa941212@</t>
-  </si>
-  <si>
-    <t>蔣耀德</t>
-  </si>
-  <si>
-    <t>password:Danny48096</t>
-  </si>
-  <si>
     <t>林恩佑</t>
   </si>
   <si>
     <t>as2d34fg</t>
   </si>
   <si>
-    <t>鄭勤翰</t>
-  </si>
-  <si>
-    <t>2945Chad</t>
-  </si>
-  <si>
     <t>藍志光</t>
   </si>
   <si>
     <t>Light0126!</t>
   </si>
   <si>
-    <t>黃謙儒</t>
-  </si>
-  <si>
-    <t>113409021ec</t>
-  </si>
-  <si>
-    <t>林季佳</t>
-  </si>
-  <si>
     <t>柯鈞泰</t>
   </si>
   <si>
-    <t>statis409023!</t>
+    <t>statis409023</t>
   </si>
   <si>
     <t>陳遠政</t>
   </si>
   <si>
-    <t>Ting0000</t>
+    <t>20041130</t>
   </si>
   <si>
     <t>陳俊宏</t>
   </si>
   <si>
-    <t>tjh13579</t>
+    <t>549221</t>
   </si>
   <si>
     <t>詹旭家</t>
@@ -551,15 +623,6 @@
     <t>葉智丞</t>
   </si>
   <si>
-    <t>NCUECO113409204</t>
-  </si>
-  <si>
-    <t>陳思璇</t>
-  </si>
-  <si>
-    <t>ophelia070907</t>
-  </si>
-  <si>
     <t>113409504</t>
   </si>
   <si>
@@ -569,91 +632,34 @@
     <t>hueicih505</t>
   </si>
   <si>
-    <t>江依霓</t>
-  </si>
-  <si>
-    <t>Xncy36</t>
-  </si>
-  <si>
-    <t>張瑋庭</t>
-  </si>
-  <si>
-    <t>Wei_815</t>
-  </si>
-  <si>
-    <t>王葦羚</t>
-  </si>
-  <si>
-    <t>lin444</t>
-  </si>
-  <si>
     <t>許馨云</t>
   </si>
   <si>
     <t>113409511113409511</t>
   </si>
   <si>
-    <t>謝宜臻</t>
-  </si>
-  <si>
-    <t>ayj901</t>
-  </si>
-  <si>
     <t>羅　萱</t>
   </si>
   <si>
-    <t>ss273027</t>
-  </si>
-  <si>
-    <t>陳宣綾</t>
-  </si>
-  <si>
-    <t>11340951870830</t>
-  </si>
-  <si>
     <t>陳彤恩</t>
   </si>
   <si>
-    <t>Ns02kety</t>
-  </si>
-  <si>
-    <t>黃妍晰</t>
-  </si>
-  <si>
-    <t>hcc7733</t>
-  </si>
-  <si>
     <t>孫偉傑</t>
   </si>
   <si>
-    <t>學生:孫偉傑
-學號:113409523
-系級:經濟二
-Password:A1234A058z</t>
+    <t>asd336e10121314</t>
   </si>
   <si>
     <t>黃政捷</t>
   </si>
   <si>
-    <t>Aa95626</t>
-  </si>
-  <si>
-    <t>蔡晟郁</t>
-  </si>
-  <si>
-    <t>20050914113409526</t>
-  </si>
-  <si>
     <t>吳淵霖</t>
   </si>
   <si>
-    <t>wendy20051222</t>
-  </si>
-  <si>
     <t>楊子逸</t>
   </si>
   <si>
-    <t>Yzy141205</t>
+    <t>29661102</t>
   </si>
   <si>
     <t>莊佑榤</t>
@@ -668,12 +674,6 @@
     <t>qwe85166517</t>
   </si>
   <si>
-    <t>江威緻</t>
-  </si>
-  <si>
-    <t>mimi0315</t>
-  </si>
-  <si>
     <t>鄭宇軒</t>
   </si>
   <si>
@@ -683,15 +683,12 @@
     <t>58706072</t>
   </si>
   <si>
-    <t>董謙耀</t>
-  </si>
-  <si>
-    <t>danny14786245</t>
-  </si>
-  <si>
     <t>文全美</t>
   </si>
   <si>
+    <t>Ria127@$</t>
+  </si>
+  <si>
     <t>連乃儀</t>
   </si>
   <si>
@@ -701,169 +698,7 @@
     <t>翁祺鈞</t>
   </si>
   <si>
-    <t>楊佳萍</t>
-  </si>
-  <si>
-    <t>Stats12345678</t>
-  </si>
-  <si>
-    <t>楊力寯</t>
-  </si>
-  <si>
-    <t>松本真裕子</t>
-  </si>
-  <si>
-    <t>阮重勝</t>
-  </si>
-  <si>
-    <t>Jdbdjddj616</t>
-  </si>
-  <si>
-    <t>陳德</t>
-  </si>
-  <si>
-    <t>password : dave060613</t>
-  </si>
-  <si>
-    <t>艾力</t>
-  </si>
-  <si>
-    <t>陳勳</t>
-  </si>
-  <si>
-    <t>劉雯惠</t>
-  </si>
-  <si>
-    <t>password:karenzacantik2104</t>
-  </si>
-  <si>
-    <t>吳榮臻</t>
-  </si>
-  <si>
-    <t>潘順財</t>
-  </si>
-  <si>
-    <t>譚浩賢</t>
-  </si>
-  <si>
-    <t>Dw089457</t>
-  </si>
-  <si>
-    <t>沈書宇</t>
-  </si>
-  <si>
-    <t>060627</t>
-  </si>
-  <si>
-    <t>中舘季来</t>
-  </si>
-  <si>
-    <t>Nakadate731</t>
-  </si>
-  <si>
-    <t>月鑽</t>
-  </si>
-  <si>
-    <t>Kaopoon.tmk06</t>
-  </si>
-  <si>
-    <t>陳慧芳</t>
-  </si>
-  <si>
-    <t>邱曉涵</t>
-  </si>
-  <si>
-    <t>陳慧晶</t>
-  </si>
-  <si>
-    <t>r3v1val15n0w</t>
-  </si>
-  <si>
-    <t>濱中芽依</t>
-  </si>
-  <si>
-    <t>mona1118</t>
-  </si>
-  <si>
-    <t>關川愛真</t>
-  </si>
-  <si>
-    <t>Emmarose0417</t>
-  </si>
-  <si>
-    <t>黄恩斯</t>
-  </si>
-  <si>
-    <t>任紹軒</t>
-  </si>
-  <si>
-    <t>faiz2525</t>
-  </si>
-  <si>
-    <t>陳義範</t>
-  </si>
-  <si>
-    <t>intake2025</t>
-  </si>
-  <si>
-    <t>陳漢亮</t>
-  </si>
-  <si>
-    <t>馮明凱</t>
-  </si>
-  <si>
-    <t>michael2025</t>
-  </si>
-  <si>
-    <t>葉明煜</t>
-  </si>
-  <si>
-    <t>蘇春福</t>
-  </si>
-  <si>
-    <t>Qwerty0909</t>
-  </si>
-  <si>
-    <t>上里苺葉</t>
-  </si>
-  <si>
-    <t>thisyeartwenty</t>
-  </si>
-  <si>
-    <t>周榮仙</t>
-  </si>
-  <si>
-    <t>鐘怡柔</t>
-  </si>
-  <si>
-    <t>Phuong@109</t>
-  </si>
-  <si>
-    <t>王祿康</t>
-  </si>
-  <si>
-    <t>lukikyn</t>
-  </si>
-  <si>
-    <t>李健明</t>
-  </si>
-  <si>
-    <t>intak2025</t>
-  </si>
-  <si>
-    <t>鄧美玲</t>
-  </si>
-  <si>
-    <t>丁聖曦</t>
-  </si>
-  <si>
-    <t>呂玟萱</t>
-  </si>
-  <si>
-    <t>徐瑋伶</t>
-  </si>
-  <si>
-    <t>許恒瑄</t>
+    <t>朱珊瑩</t>
   </si>
   <si>
     <t>Olivia</t>
@@ -912,7 +747,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -924,6 +759,8 @@
       <b/>
       <sz val="11"/>
       <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
     </font>
     <font>
       <sz val="9"/>
@@ -931,6 +768,11 @@
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="新細明體"/>
     </font>
   </fonts>
   <fills count="2">
@@ -941,7 +783,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -971,13 +813,34 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1282,216 +1145,216 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>110408547</v>
+        <v>110408302</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
+        <v>60</v>
+      </c>
+      <c r="C2">
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>112103011</v>
+        <v>110408527</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>112602527</v>
+        <v>112103011</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4">
-        <v>123</v>
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>113401526</v>
+        <v>112408003</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>113408001</v>
+        <v>113401526</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>113408002</v>
+        <v>113408001</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>113408003</v>
+        <v>113408002</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>113408004</v>
+        <v>113408003</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>113408005</v>
+        <v>113408004</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>113408007</v>
+        <v>113408005</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
+        <v>77</v>
+      </c>
+      <c r="C11">
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>113408008</v>
+        <v>113408007</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>113408009</v>
+        <v>113408008</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13">
-        <v>123</v>
+        <v>80</v>
+      </c>
+      <c r="C13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>113408010</v>
+        <v>113408009</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>113408011</v>
+        <v>113408010</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>113408012</v>
+        <v>113408011</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>113408015</v>
+        <v>113408012</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" t="s">
-        <v>32</v>
+        <v>88</v>
+      </c>
+      <c r="C17">
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>113408016</v>
+        <v>113408015</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>113408017</v>
+        <v>113408016</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -1499,10 +1362,10 @@
         <v>113408018</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -1510,10 +1373,10 @@
         <v>113408019</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -1521,10 +1384,10 @@
         <v>113408020</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22">
-        <v>123</v>
+        <v>97</v>
+      </c>
+      <c r="C22" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -1532,10 +1395,10 @@
         <v>113408022</v>
       </c>
       <c r="B23" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -1543,10 +1406,10 @@
         <v>113408025</v>
       </c>
       <c r="B24" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -1554,10 +1417,10 @@
         <v>113408027</v>
       </c>
       <c r="B25" t="s">
-        <v>46</v>
+        <v>103</v>
       </c>
       <c r="C25" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -1565,10 +1428,10 @@
         <v>113408028</v>
       </c>
       <c r="B26" t="s">
-        <v>48</v>
+        <v>105</v>
       </c>
       <c r="C26" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -1576,10 +1439,10 @@
         <v>113408030</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
+        <v>107</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -1587,7 +1450,7 @@
         <v>113408201</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>109</v>
       </c>
       <c r="C28">
         <v>123</v>
@@ -1598,10 +1461,10 @@
         <v>113408501</v>
       </c>
       <c r="B29" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -1609,10 +1472,10 @@
         <v>113408502</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>112</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -1620,10 +1483,10 @@
         <v>113408503</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>114</v>
       </c>
       <c r="C31" t="s">
-        <v>58</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -1631,10 +1494,10 @@
         <v>113408504</v>
       </c>
       <c r="B32" t="s">
-        <v>59</v>
+        <v>116</v>
       </c>
       <c r="C32" t="s">
-        <v>60</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -1642,10 +1505,10 @@
         <v>113408505</v>
       </c>
       <c r="B33" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
       <c r="C33" t="s">
-        <v>62</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -1653,10 +1516,10 @@
         <v>113408506</v>
       </c>
       <c r="B34" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="C34" t="s">
-        <v>64</v>
+        <v>121</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -1664,10 +1527,10 @@
         <v>113408507</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>122</v>
       </c>
       <c r="C35" t="s">
-        <v>66</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -1675,10 +1538,10 @@
         <v>113408508</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>125</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -1686,10 +1549,10 @@
         <v>113408509</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>126</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>127</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -1697,10 +1560,10 @@
         <v>113408510</v>
       </c>
       <c r="B38" t="s">
-        <v>71</v>
+        <v>128</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -1708,10 +1571,10 @@
         <v>113408511</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>131</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -1719,10 +1582,10 @@
         <v>113408512</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>132</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
+        <v>133</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -1730,10 +1593,10 @@
         <v>113408513</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>134</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
+        <v>135</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -1741,10 +1604,10 @@
         <v>113408514</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>136</v>
       </c>
       <c r="C42" t="s">
-        <v>80</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -1752,10 +1615,10 @@
         <v>113408515</v>
       </c>
       <c r="B43" t="s">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="C43" t="s">
-        <v>82</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -1763,10 +1626,10 @@
         <v>113408516</v>
       </c>
       <c r="B44" t="s">
-        <v>83</v>
+        <v>140</v>
       </c>
       <c r="C44" t="s">
-        <v>84</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -1774,10 +1637,10 @@
         <v>113408517</v>
       </c>
       <c r="B45" t="s">
-        <v>85</v>
+        <v>142</v>
       </c>
       <c r="C45" t="s">
-        <v>86</v>
+        <v>143</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -1785,10 +1648,10 @@
         <v>113408518</v>
       </c>
       <c r="B46" t="s">
-        <v>87</v>
+        <v>144</v>
       </c>
       <c r="C46" t="s">
-        <v>88</v>
+        <v>145</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -1796,10 +1659,10 @@
         <v>113408519</v>
       </c>
       <c r="B47" t="s">
-        <v>89</v>
+        <v>146</v>
       </c>
       <c r="C47" t="s">
-        <v>90</v>
+        <v>147</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -1807,10 +1670,10 @@
         <v>113408520</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="C48" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -1818,10 +1681,10 @@
         <v>113408521</v>
       </c>
       <c r="B49" t="s">
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="C49" t="s">
-        <v>94</v>
+        <v>151</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -1829,10 +1692,10 @@
         <v>113408522</v>
       </c>
       <c r="B50" t="s">
-        <v>95</v>
+        <v>152</v>
       </c>
       <c r="C50" t="s">
-        <v>96</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -1840,10 +1703,10 @@
         <v>113408523</v>
       </c>
       <c r="B51" t="s">
-        <v>97</v>
+        <v>154</v>
       </c>
       <c r="C51" t="s">
-        <v>98</v>
+        <v>155</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -1851,10 +1714,10 @@
         <v>113408525</v>
       </c>
       <c r="B52" t="s">
-        <v>99</v>
+        <v>156</v>
       </c>
       <c r="C52" t="s">
-        <v>100</v>
+        <v>157</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -1862,7 +1725,7 @@
         <v>113408526</v>
       </c>
       <c r="B53" t="s">
-        <v>101</v>
+        <v>158</v>
       </c>
       <c r="C53">
         <v>123</v>
@@ -1873,10 +1736,10 @@
         <v>113408527</v>
       </c>
       <c r="B54" t="s">
-        <v>102</v>
+        <v>159</v>
       </c>
       <c r="C54" t="s">
-        <v>103</v>
+        <v>160</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -1884,10 +1747,10 @@
         <v>113408528</v>
       </c>
       <c r="B55" t="s">
-        <v>104</v>
+        <v>161</v>
       </c>
       <c r="C55" t="s">
-        <v>105</v>
+        <v>162</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -1895,10 +1758,10 @@
         <v>113408529</v>
       </c>
       <c r="B56" t="s">
-        <v>106</v>
+        <v>163</v>
       </c>
       <c r="C56" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
@@ -1906,29 +1769,29 @@
         <v>113408530</v>
       </c>
       <c r="B57" t="s">
-        <v>108</v>
-      </c>
-      <c r="C57" t="s">
-        <v>109</v>
+        <v>165</v>
+      </c>
+      <c r="C57">
+        <v>123</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>113408531</v>
+        <v>113408533</v>
       </c>
       <c r="B58" t="s">
-        <v>110</v>
-      </c>
-      <c r="C58" t="s">
-        <v>111</v>
+        <v>166</v>
+      </c>
+      <c r="C58">
+        <v>123</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>113408532</v>
+        <v>113408534</v>
       </c>
       <c r="B59" t="s">
-        <v>112</v>
+        <v>167</v>
       </c>
       <c r="C59">
         <v>123</v>
@@ -1936,54 +1799,54 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>113408533</v>
+        <v>113408535</v>
       </c>
       <c r="B60" t="s">
-        <v>113</v>
-      </c>
-      <c r="C60" t="s">
-        <v>114</v>
+        <v>168</v>
+      </c>
+      <c r="C60">
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>113408534</v>
+        <v>113707517</v>
       </c>
       <c r="B61" t="s">
-        <v>115</v>
-      </c>
-      <c r="C61" t="s">
-        <v>116</v>
+        <v>169</v>
+      </c>
+      <c r="C61">
+        <v>123</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>113408535</v>
+        <v>110102007</v>
       </c>
       <c r="B62" t="s">
-        <v>117</v>
-      </c>
-      <c r="C62" t="s">
-        <v>118</v>
+        <v>170</v>
+      </c>
+      <c r="C62">
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>113707517</v>
+        <v>112102525</v>
       </c>
       <c r="B63" t="s">
-        <v>119</v>
-      </c>
-      <c r="C63" t="s">
-        <v>120</v>
+        <v>171</v>
+      </c>
+      <c r="C63">
+        <v>123</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>111408510</v>
+        <v>111408531</v>
       </c>
       <c r="B64" t="s">
-        <v>121</v>
+        <v>172</v>
       </c>
       <c r="C64">
         <v>123</v>
@@ -1991,13 +1854,24 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>112408024</v>
+        <v>112408501</v>
       </c>
       <c r="B65" t="s">
-        <v>122</v>
+        <v>173</v>
       </c>
       <c r="C65">
         <v>123</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>8142122</v>
+      </c>
+      <c r="B66" t="s">
+        <v>174</v>
+      </c>
+      <c r="C66">
+        <v>8142122</v>
       </c>
     </row>
   </sheetData>
@@ -2008,26 +1882,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>109401533</v>
+        <v>112409020</v>
       </c>
       <c r="B2" t="s">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="C2">
         <v>123</v>
@@ -2035,21 +1909,21 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>111103514</v>
+        <v>113102007</v>
       </c>
       <c r="B3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C3">
-        <v>123</v>
+        <v>176</v>
+      </c>
+      <c r="C3" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>112101003</v>
+        <v>113409004</v>
       </c>
       <c r="B4" t="s">
-        <v>125</v>
+        <v>178</v>
       </c>
       <c r="C4">
         <v>123</v>
@@ -2057,585 +1931,321 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>112102525</v>
+        <v>113409006</v>
       </c>
       <c r="B5" t="s">
-        <v>126</v>
+        <v>179</v>
       </c>
       <c r="C5" t="s">
-        <v>127</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>112409020</v>
+        <v>113409009</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
-      </c>
-      <c r="C6">
-        <v>123</v>
+        <v>181</v>
+      </c>
+      <c r="C6" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>112707001</v>
+        <v>113409011</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C7" t="s">
-        <v>130</v>
+        <v>183</v>
+      </c>
+      <c r="C7">
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>112707508</v>
+        <v>113409013</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C8" t="s">
-        <v>132</v>
+        <v>184</v>
+      </c>
+      <c r="C8">
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>113102007</v>
+        <v>113409015</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
-      </c>
-      <c r="C9" t="s">
-        <v>134</v>
+        <v>185</v>
+      </c>
+      <c r="C9">
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>113409001</v>
+        <v>113409017</v>
       </c>
       <c r="B10" t="s">
-        <v>135</v>
+        <v>186</v>
       </c>
       <c r="C10" t="s">
-        <v>136</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>113409004</v>
+        <v>113409020</v>
       </c>
       <c r="B11" t="s">
-        <v>137</v>
+        <v>188</v>
       </c>
       <c r="C11" t="s">
-        <v>138</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>113409005</v>
+        <v>113409023</v>
       </c>
       <c r="B12" t="s">
-        <v>139</v>
-      </c>
-      <c r="C12">
-        <v>123</v>
+        <v>190</v>
+      </c>
+      <c r="C12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>113409006</v>
+        <v>113409024</v>
       </c>
       <c r="B13" t="s">
-        <v>140</v>
+        <v>192</v>
       </c>
       <c r="C13" t="s">
-        <v>141</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>113409008</v>
+        <v>113409025</v>
       </c>
       <c r="B14" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C14" t="s">
-        <v>143</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>113409009</v>
+        <v>113409026</v>
       </c>
       <c r="B15" t="s">
-        <v>144</v>
+        <v>196</v>
       </c>
       <c r="C15" t="s">
-        <v>145</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>113409011</v>
+        <v>113409204</v>
       </c>
       <c r="B16" t="s">
-        <v>146</v>
-      </c>
-      <c r="C16" t="s">
-        <v>147</v>
+        <v>198</v>
+      </c>
+      <c r="C16">
+        <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>113409012</v>
+        <v>113409504</v>
       </c>
       <c r="B17" t="s">
-        <v>148</v>
-      </c>
-      <c r="C17">
-        <v>123</v>
+        <v>138</v>
+      </c>
+      <c r="C17" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>113409013</v>
+        <v>113409505</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>200</v>
       </c>
       <c r="C18" t="s">
-        <v>150</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>113409014</v>
+        <v>113409511</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>202</v>
       </c>
       <c r="C19" t="s">
-        <v>152</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>113409015</v>
+        <v>113409513</v>
       </c>
       <c r="B20" t="s">
-        <v>153</v>
-      </c>
-      <c r="C20" t="s">
-        <v>154</v>
+        <v>204</v>
+      </c>
+      <c r="C20">
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>113409016</v>
+        <v>113409519</v>
       </c>
       <c r="B21" t="s">
-        <v>155</v>
-      </c>
-      <c r="C21" t="s">
-        <v>156</v>
+        <v>205</v>
+      </c>
+      <c r="C21">
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>113409017</v>
+        <v>113409523</v>
       </c>
       <c r="B22" t="s">
-        <v>157</v>
+        <v>206</v>
       </c>
       <c r="C22" t="s">
-        <v>158</v>
+        <v>207</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>113409019</v>
+        <v>113409525</v>
       </c>
       <c r="B23" t="s">
-        <v>159</v>
-      </c>
-      <c r="C23" t="s">
-        <v>160</v>
+        <v>208</v>
+      </c>
+      <c r="C23">
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>113409020</v>
+        <v>113409527</v>
       </c>
       <c r="B24" t="s">
-        <v>161</v>
-      </c>
-      <c r="C24" t="s">
-        <v>162</v>
+        <v>209</v>
+      </c>
+      <c r="C24">
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>113409021</v>
+        <v>113409529</v>
       </c>
       <c r="B25" t="s">
-        <v>163</v>
+        <v>210</v>
       </c>
       <c r="C25" t="s">
-        <v>164</v>
+        <v>211</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>113409022</v>
+        <v>113409530</v>
       </c>
       <c r="B26" t="s">
-        <v>165</v>
-      </c>
-      <c r="C26">
-        <v>123</v>
+        <v>212</v>
+      </c>
+      <c r="C26" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>113409023</v>
+        <v>113409532</v>
       </c>
       <c r="B27" t="s">
-        <v>166</v>
+        <v>214</v>
       </c>
       <c r="C27" t="s">
-        <v>167</v>
+        <v>215</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>113409024</v>
+        <v>113409536</v>
       </c>
       <c r="B28" t="s">
-        <v>168</v>
-      </c>
-      <c r="C28" t="s">
-        <v>169</v>
+        <v>216</v>
+      </c>
+      <c r="C28">
+        <v>123</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>113409025</v>
+        <v>113409537</v>
       </c>
       <c r="B29" t="s">
-        <v>170</v>
+        <v>217</v>
       </c>
       <c r="C29" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>113409026</v>
+        <v>113409601</v>
       </c>
       <c r="B30" t="s">
-        <v>172</v>
+        <v>219</v>
       </c>
       <c r="C30" t="s">
-        <v>173</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>113409204</v>
+        <v>113707519</v>
       </c>
       <c r="B31" t="s">
-        <v>174</v>
+        <v>221</v>
       </c>
       <c r="C31" t="s">
-        <v>175</v>
+        <v>222</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>113409502</v>
+        <v>112502533</v>
       </c>
       <c r="B32" t="s">
-        <v>176</v>
-      </c>
-      <c r="C32" t="s">
-        <v>177</v>
+        <v>223</v>
+      </c>
+      <c r="C32">
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>113409504</v>
+        <v>11772</v>
       </c>
       <c r="B33" t="s">
-        <v>81</v>
-      </c>
-      <c r="C33" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>113409505</v>
-      </c>
-      <c r="B34" t="s">
-        <v>179</v>
-      </c>
-      <c r="C34" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>113409508</v>
-      </c>
-      <c r="B35" t="s">
-        <v>181</v>
-      </c>
-      <c r="C35" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>113409509</v>
-      </c>
-      <c r="B36" t="s">
-        <v>183</v>
-      </c>
-      <c r="C36" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>113409510</v>
-      </c>
-      <c r="B37" t="s">
-        <v>185</v>
-      </c>
-      <c r="C37" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>113409511</v>
-      </c>
-      <c r="B38" t="s">
-        <v>187</v>
-      </c>
-      <c r="C38" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>113409512</v>
-      </c>
-      <c r="B39" t="s">
-        <v>189</v>
-      </c>
-      <c r="C39" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40">
-        <v>113409513</v>
-      </c>
-      <c r="B40" t="s">
-        <v>191</v>
-      </c>
-      <c r="C40" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41">
-        <v>113409518</v>
-      </c>
-      <c r="B41" t="s">
-        <v>193</v>
-      </c>
-      <c r="C41" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42">
-        <v>113409519</v>
-      </c>
-      <c r="B42" t="s">
-        <v>195</v>
-      </c>
-      <c r="C42" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43">
-        <v>113409520</v>
-      </c>
-      <c r="B43" t="s">
-        <v>197</v>
-      </c>
-      <c r="C43" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44">
-        <v>113409523</v>
-      </c>
-      <c r="B44" t="s">
-        <v>199</v>
-      </c>
-      <c r="C44" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45">
-        <v>113409525</v>
-      </c>
-      <c r="B45" t="s">
-        <v>201</v>
-      </c>
-      <c r="C45" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46">
-        <v>113409526</v>
-      </c>
-      <c r="B46" t="s">
-        <v>203</v>
-      </c>
-      <c r="C46" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47">
-        <v>113409527</v>
-      </c>
-      <c r="B47" t="s">
-        <v>205</v>
-      </c>
-      <c r="C47" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48">
-        <v>113409529</v>
-      </c>
-      <c r="B48" t="s">
-        <v>207</v>
-      </c>
-      <c r="C48" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49">
-        <v>113409530</v>
-      </c>
-      <c r="B49" t="s">
-        <v>209</v>
-      </c>
-      <c r="C49" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50">
-        <v>113409532</v>
-      </c>
-      <c r="B50" t="s">
-        <v>211</v>
-      </c>
-      <c r="C50" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51">
-        <v>113409535</v>
-      </c>
-      <c r="B51" t="s">
-        <v>213</v>
-      </c>
-      <c r="C51" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52">
-        <v>113409536</v>
-      </c>
-      <c r="B52" t="s">
-        <v>215</v>
-      </c>
-      <c r="C52">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53">
-        <v>113409537</v>
-      </c>
-      <c r="B53" t="s">
-        <v>216</v>
-      </c>
-      <c r="C53" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54">
-        <v>113409538</v>
-      </c>
-      <c r="B54" t="s">
-        <v>218</v>
-      </c>
-      <c r="C54" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55">
-        <v>113409601</v>
-      </c>
-      <c r="B55" t="s">
-        <v>220</v>
-      </c>
-      <c r="C55">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56">
-        <v>113707519</v>
-      </c>
-      <c r="B56" t="s">
-        <v>221</v>
-      </c>
-      <c r="C56" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57">
-        <v>112502533</v>
-      </c>
-      <c r="B57" t="s">
-        <v>223</v>
-      </c>
-      <c r="C57">
-        <v>123</v>
+        <v>224</v>
+      </c>
+      <c r="C33">
+        <v>11772</v>
       </c>
     </row>
   </sheetData>
@@ -2646,8 +2256,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -2661,308 +2274,308 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>11140294</v>
-      </c>
-      <c r="B2" t="s">
-        <v>224</v>
-      </c>
-      <c r="C2" t="s">
-        <v>225</v>
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>11149171</v>
-      </c>
-      <c r="B3" t="s">
-        <v>226</v>
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="C3">
         <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>11240277</v>
-      </c>
-      <c r="B4" t="s">
-        <v>227</v>
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="C4">
         <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>11240297</v>
-      </c>
-      <c r="B5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C5" t="s">
-        <v>229</v>
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>11240300</v>
-      </c>
-      <c r="B6" t="s">
-        <v>230</v>
-      </c>
-      <c r="C6" t="s">
-        <v>231</v>
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>11240307</v>
-      </c>
-      <c r="B7" t="s">
-        <v>232</v>
+      <c r="A7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="C7">
         <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>11240316</v>
-      </c>
-      <c r="B8" t="s">
-        <v>233</v>
+      <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C8">
         <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>11340171</v>
-      </c>
-      <c r="B9" t="s">
-        <v>234</v>
-      </c>
-      <c r="C9" t="s">
-        <v>235</v>
+      <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9">
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>11340172</v>
-      </c>
-      <c r="B10" t="s">
-        <v>236</v>
+      <c r="A10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="C10">
         <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>11340173</v>
-      </c>
-      <c r="B11" t="s">
-        <v>237</v>
+      <c r="A11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="C11">
         <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>11340174</v>
-      </c>
-      <c r="B12" t="s">
-        <v>238</v>
-      </c>
-      <c r="C12" t="s">
-        <v>239</v>
+      <c r="A12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12">
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>11340175</v>
-      </c>
-      <c r="B13" t="s">
-        <v>240</v>
-      </c>
-      <c r="C13" t="s">
-        <v>241</v>
+      <c r="A13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13">
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>11340179</v>
-      </c>
-      <c r="B14" t="s">
-        <v>242</v>
-      </c>
-      <c r="C14" t="s">
-        <v>243</v>
+      <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14">
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>11340180</v>
-      </c>
-      <c r="B15" t="s">
-        <v>244</v>
-      </c>
-      <c r="C15" t="s">
-        <v>245</v>
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15">
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>11340184</v>
-      </c>
-      <c r="B16" t="s">
-        <v>246</v>
+      <c r="A16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="C16">
         <v>123</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>11340188</v>
-      </c>
-      <c r="B17" t="s">
-        <v>247</v>
+      <c r="A17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="C17">
         <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>11340192</v>
-      </c>
-      <c r="B18" t="s">
-        <v>248</v>
-      </c>
-      <c r="C18" t="s">
-        <v>249</v>
+      <c r="A18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18">
+        <v>123</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>11340197</v>
-      </c>
-      <c r="B19" t="s">
-        <v>250</v>
-      </c>
-      <c r="C19" t="s">
-        <v>251</v>
+      <c r="A19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19">
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>11340198</v>
-      </c>
-      <c r="B20" t="s">
-        <v>252</v>
-      </c>
-      <c r="C20" t="s">
-        <v>253</v>
+      <c r="A20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20">
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>11340199</v>
-      </c>
-      <c r="B21" t="s">
-        <v>254</v>
+      <c r="A21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="C21">
         <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>11340201</v>
-      </c>
-      <c r="B22" t="s">
-        <v>255</v>
-      </c>
-      <c r="C22" t="s">
-        <v>256</v>
+      <c r="A22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22">
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>11340209</v>
-      </c>
-      <c r="B23" t="s">
-        <v>257</v>
-      </c>
-      <c r="C23" t="s">
-        <v>258</v>
+      <c r="A23" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23">
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>11340210</v>
-      </c>
-      <c r="B24" t="s">
-        <v>259</v>
+      <c r="A24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="C24">
         <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>11340215</v>
-      </c>
-      <c r="B25" t="s">
-        <v>260</v>
-      </c>
-      <c r="C25" t="s">
-        <v>261</v>
+      <c r="A25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25">
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>11340217</v>
-      </c>
-      <c r="B26" t="s">
-        <v>262</v>
+      <c r="A26" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="C26">
         <v>123</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>11340219</v>
-      </c>
-      <c r="B27" t="s">
-        <v>263</v>
-      </c>
-      <c r="C27" t="s">
-        <v>264</v>
+      <c r="A27" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27">
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>11340220</v>
-      </c>
-      <c r="B28" t="s">
-        <v>265</v>
-      </c>
-      <c r="C28" t="s">
-        <v>266</v>
+      <c r="A28" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28">
+        <v>123</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>11340222</v>
-      </c>
-      <c r="B29" t="s">
-        <v>267</v>
+      <c r="A29" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="C29">
         <v>123</v>
@@ -2970,89 +2583,12 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>11340230</v>
-      </c>
-      <c r="B30" t="s">
-        <v>268</v>
-      </c>
-      <c r="C30" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>11340231</v>
-      </c>
-      <c r="B31" t="s">
-        <v>270</v>
-      </c>
-      <c r="C31" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>11340232</v>
-      </c>
-      <c r="B32" t="s">
-        <v>272</v>
-      </c>
-      <c r="C32" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>11340233</v>
-      </c>
-      <c r="B33" t="s">
-        <v>274</v>
-      </c>
-      <c r="C33">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34">
         <v>11344114</v>
       </c>
-      <c r="B34" t="s">
-        <v>275</v>
-      </c>
-      <c r="C34">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>11141206</v>
-      </c>
-      <c r="B35" t="s">
-        <v>276</v>
-      </c>
-      <c r="C35">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>11241419</v>
-      </c>
-      <c r="B36" t="s">
-        <v>277</v>
-      </c>
-      <c r="C36">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>11241422</v>
-      </c>
-      <c r="B37" t="s">
-        <v>278</v>
-      </c>
-      <c r="C37">
+      <c r="B30" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30">
         <v>123</v>
       </c>
     </row>
@@ -3063,7 +2599,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F457DE-58B8-40BD-8914-8E21464647DB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -3083,7 +2619,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>279</v>
+        <v>225</v>
       </c>
       <c r="C2">
         <v>123</v>
@@ -3094,7 +2630,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>280</v>
+        <v>226</v>
       </c>
       <c r="C3">
         <v>123</v>
@@ -3105,7 +2641,7 @@
         <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>281</v>
+        <v>227</v>
       </c>
       <c r="C4">
         <v>123</v>
@@ -3116,7 +2652,7 @@
         <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>282</v>
+        <v>228</v>
       </c>
       <c r="C5">
         <v>123</v>
@@ -3127,7 +2663,7 @@
         <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>283</v>
+        <v>229</v>
       </c>
       <c r="C6">
         <v>123</v>
@@ -3138,7 +2674,7 @@
         <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>284</v>
+        <v>230</v>
       </c>
       <c r="C7">
         <v>123</v>
@@ -3149,7 +2685,7 @@
         <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>285</v>
+        <v>231</v>
       </c>
       <c r="C8">
         <v>123</v>
@@ -3160,7 +2696,7 @@
         <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>286</v>
+        <v>232</v>
       </c>
       <c r="C9">
         <v>123</v>
@@ -3171,7 +2707,7 @@
         <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>287</v>
+        <v>233</v>
       </c>
       <c r="C10">
         <v>123</v>
@@ -3182,7 +2718,7 @@
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>288</v>
+        <v>234</v>
       </c>
       <c r="C11">
         <v>123</v>
@@ -3193,7 +2729,7 @@
         <v>111</v>
       </c>
       <c r="B12" t="s">
-        <v>289</v>
+        <v>235</v>
       </c>
       <c r="C12">
         <v>123</v>
@@ -3204,7 +2740,7 @@
         <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>290</v>
+        <v>236</v>
       </c>
       <c r="C13">
         <v>123</v>
@@ -3215,7 +2751,7 @@
         <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>291</v>
+        <v>237</v>
       </c>
       <c r="C14">
         <v>123</v>
@@ -3226,7 +2762,7 @@
         <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>292</v>
+        <v>238</v>
       </c>
       <c r="C15">
         <v>123</v>

</xml_diff>